<commit_message>
feat: added gsheet and brevo cloud email api
</commit_message>
<xml_diff>
--- a/backend/bookings.xlsx
+++ b/backend/bookings.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -573,6 +573,46 @@
         </is>
       </c>
       <c r="H4" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>5</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-09-21 15:40:03</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Medicine Delivery</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Aman Haz</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>6002323454</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>rupankarb1@gmail.com</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Delivery address: Siliguri; Medicines: nnn; Preferred delivery date: 2026-09-23</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
         <is>
           <t>Confirmed</t>
         </is>

</xml_diff>